<commit_message>
update 9 combinations benchmark and resource estimation
</commit_message>
<xml_diff>
--- a/output/benchmark_data_dataset_A_COBYLA_vs_back-propagate.xlsx
+++ b/output/benchmark_data_dataset_A_COBYLA_vs_back-propagate.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,22 +566,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>-633.5514108391153</v>
+        <v>-633.4968349180199</v>
       </c>
       <c r="C2" t="n">
-        <v>1.013781255413816</v>
+        <v>1.169851034049424</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1998898205074298</v>
+        <v>-0.5228349072079568</v>
       </c>
       <c r="E2" t="n">
-        <v>-580.7642788262604</v>
+        <v>-653.1536284759719</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8708242505446556</v>
+        <v>0.9571499291696618</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.3974762026007553</v>
+        <v>0.07213252579736437</v>
       </c>
     </row>
     <row r="3">
@@ -589,22 +589,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>-698.6606537966378</v>
+        <v>-667.1871280104209</v>
       </c>
       <c r="C3" t="n">
-        <v>1.322942941768214</v>
+        <v>1.353271002894624</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1311405139113197</v>
+        <v>-0.6025664256233599</v>
       </c>
       <c r="E3" t="n">
-        <v>-640.7739934225061</v>
+        <v>-690.3571505588509</v>
       </c>
       <c r="F3" t="n">
-        <v>0.772612237304277</v>
+        <v>0.9571499291696618</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.378650675907679</v>
+        <v>0.07213252579736437</v>
       </c>
     </row>
     <row r="4">
@@ -612,22 +612,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>-702.4743235338707</v>
+        <v>-667.1871280104209</v>
       </c>
       <c r="C4" t="n">
-        <v>1.470516226720223</v>
+        <v>1.353271002894624</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.003848839626184253</v>
+        <v>-0.6025664256233599</v>
       </c>
       <c r="E4" t="n">
-        <v>-672.5045712547571</v>
+        <v>-698.4077049772762</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7185144300150078</v>
+        <v>0.9571499291696618</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.4053231452203878</v>
+        <v>0.07213252579736437</v>
       </c>
     </row>
     <row r="5">
@@ -635,22 +635,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>-711.9788604966267</v>
+        <v>-685.6887119483075</v>
       </c>
       <c r="C5" t="n">
-        <v>1.8151404384592</v>
+        <v>1.335697252712408</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.01215188318925997</v>
+        <v>-0.6121143732841443</v>
       </c>
       <c r="E5" t="n">
-        <v>-672.5045712547571</v>
+        <v>-730.0293936793917</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7185144300150078</v>
+        <v>0.9548885454016498</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.4053231452203878</v>
+        <v>0.08187347767352977</v>
       </c>
     </row>
     <row r="6">
@@ -658,22 +658,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>-733.5160911142281</v>
+        <v>-718.3611582002745</v>
       </c>
       <c r="C6" t="n">
-        <v>3.104255090996585</v>
+        <v>1.792798783186234</v>
       </c>
       <c r="D6" t="n">
-        <v>0.14685563754153</v>
+        <v>-0.7922748992106197</v>
       </c>
       <c r="E6" t="n">
-        <v>-696.3572069238853</v>
+        <v>-739.6115662272319</v>
       </c>
       <c r="F6" t="n">
-        <v>0.774512891753768</v>
+        <v>1.148876363816694</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1630757150316192</v>
+        <v>0.3286512550932764</v>
       </c>
     </row>
     <row r="7">
@@ -681,22 +681,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>-736.7208389501668</v>
+        <v>-718.3611582002745</v>
       </c>
       <c r="C7" t="n">
-        <v>4.724344792116263</v>
+        <v>1.792798783186234</v>
       </c>
       <c r="D7" t="n">
-        <v>0.37714469350668</v>
+        <v>-0.7922748992106197</v>
       </c>
       <c r="E7" t="n">
-        <v>-696.3572069238853</v>
+        <v>-791.7696721372024</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4327240994418502</v>
+        <v>1.523736808712341</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1822706035603775</v>
+        <v>1.278484359402879</v>
       </c>
     </row>
     <row r="8">
@@ -704,91 +704,17 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>-736.7208389501668</v>
+        <v>-718.3611582002745</v>
       </c>
       <c r="C8" t="n">
-        <v>4.724344792116263</v>
+        <v>2.066912004124847</v>
       </c>
       <c r="D8" t="n">
-        <v>0.37714469350668</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-696.3572069238853</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.38448201937392</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.3602470986221622</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>-736.7208389501668</v>
-      </c>
-      <c r="C9" t="n">
-        <v>4.724344792116263</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.37714469350668</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="n">
-        <v>-747.9675393158724</v>
-      </c>
-      <c r="C10" t="n">
-        <v>6.497921104387729</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2.653142568940121</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="n">
-        <v>-756.1963787438115</v>
-      </c>
-      <c r="C11" t="n">
-        <v>6.248012302130292</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2.659894646713159</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="n">
-        <v>-756.1963787438115</v>
-      </c>
-      <c r="C12" t="n">
-        <v>6.248012302130292</v>
-      </c>
-      <c r="D12" t="n">
-        <v>2.659894646713159</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+        <v>-0.1417057850253216</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -801,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C257"/>
+  <dimension ref="A1:C258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -828,10 +754,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0015625</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0021484375</v>
+        <v>0.000390625</v>
       </c>
     </row>
     <row r="3">
@@ -841,10 +767,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001953125</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0021484375</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="4">
@@ -857,7 +783,7 @@
         <v>0.00390625</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0009765625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="5">
@@ -867,10 +793,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0052734375</v>
+        <v>0.01015625</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0015625</v>
+        <v>0.005859375</v>
       </c>
     </row>
     <row r="6">
@@ -880,10 +806,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.001171875</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C6" t="n">
-        <v>0.003125</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="7">
@@ -893,10 +819,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0017578125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0033203125</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="8">
@@ -906,10 +832,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0056640625</v>
+        <v>0.003515625</v>
       </c>
       <c r="C8" t="n">
-        <v>0.001953125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="9">
@@ -919,10 +845,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.005078125</v>
+        <v>0.0029296875</v>
       </c>
       <c r="C9" t="n">
-        <v>0.003515625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="10">
@@ -932,10 +858,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0013671875</v>
+        <v>0.0015625</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0013671875</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="11">
@@ -945,10 +871,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.002734375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C11" t="n">
-        <v>0.00078125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="12">
@@ -958,10 +884,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.002734375</v>
+        <v>0.001953125</v>
       </c>
       <c r="C12" t="n">
-        <v>0.001953125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="13">
@@ -971,10 +897,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0025390625</v>
+        <v>0.0046875</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0017578125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="14">
@@ -984,10 +910,10 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>0.001171875</v>
+      </c>
+      <c r="C14" t="n">
         <v>0.0021484375</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.001171875</v>
       </c>
     </row>
     <row r="15">
@@ -997,10 +923,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0041015625</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0033203125</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="16">
@@ -1010,10 +936,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0017578125</v>
+        <v>0.001953125</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0021484375</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="17">
@@ -1023,10 +949,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0025390625</v>
+        <v>0.00234375</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0033203125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="18">
@@ -1036,10 +962,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00234375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0083984375</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="19">
@@ -1049,10 +975,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.00703125</v>
+        <v>0.0056640625</v>
       </c>
       <c r="C19" t="n">
-        <v>0.009960937499999999</v>
+        <v>0.004296875</v>
       </c>
     </row>
     <row r="20">
@@ -1062,10 +988,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.005078125</v>
+        <v>0.0046875</v>
       </c>
       <c r="C20" t="n">
-        <v>0.003515625</v>
+        <v>0.0068359375</v>
       </c>
     </row>
     <row r="21">
@@ -1075,10 +1001,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.01015625</v>
+        <v>0.0177734375</v>
       </c>
       <c r="C21" t="n">
-        <v>0.00546875</v>
+        <v>0.021875</v>
       </c>
     </row>
     <row r="22">
@@ -1088,10 +1014,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.0029296875</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C22" t="n">
-        <v>0.0037109375</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="23">
@@ -1101,7 +1027,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0021484375</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C23" t="n">
         <v>0.0021484375</v>
@@ -1114,10 +1040,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.005859375</v>
+        <v>0.003515625</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0029296875</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="25">
@@ -1127,10 +1053,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.008593750000000001</v>
+        <v>0.0125</v>
       </c>
       <c r="C25" t="n">
-        <v>0.00234375</v>
+        <v>0.005859375</v>
       </c>
     </row>
     <row r="26">
@@ -1140,10 +1066,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.0041015625</v>
+        <v>0.001953125</v>
       </c>
       <c r="C26" t="n">
-        <v>0.0056640625</v>
+        <v>0.007421875</v>
       </c>
     </row>
     <row r="27">
@@ -1153,10 +1079,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.0109375</v>
+        <v>0.005078125</v>
       </c>
       <c r="C27" t="n">
-        <v>0.00546875</v>
+        <v>0.01015625</v>
       </c>
     </row>
     <row r="28">
@@ -1166,10 +1092,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.00390625</v>
+        <v>0.0037109375</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0052734375</v>
+        <v>0.004296875</v>
       </c>
     </row>
     <row r="29">
@@ -1179,10 +1105,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.007421875</v>
+        <v>0.0177734375</v>
       </c>
       <c r="C29" t="n">
-        <v>0.009375</v>
+        <v>0.0103515625</v>
       </c>
     </row>
     <row r="30">
@@ -1192,10 +1118,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.0052734375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C30" t="n">
-        <v>0.0025390625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="31">
@@ -1205,10 +1131,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.0078125</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C31" t="n">
-        <v>0.0029296875</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="32">
@@ -1218,10 +1144,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.004296875</v>
+        <v>0.00390625</v>
       </c>
       <c r="C32" t="n">
-        <v>0.002734375</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="33">
@@ -1231,10 +1157,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.0033203125</v>
+        <v>0.0091796875</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0017578125</v>
+        <v>0.003515625</v>
       </c>
     </row>
     <row r="34">
@@ -1244,10 +1170,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.00234375</v>
+        <v>0.001953125</v>
       </c>
       <c r="C34" t="n">
-        <v>0.0009765625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="35">
@@ -1257,10 +1183,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.0033203125</v>
+        <v>0.00546875</v>
       </c>
       <c r="C35" t="n">
-        <v>0.0013671875</v>
+        <v>0.0041015625</v>
       </c>
     </row>
     <row r="36">
@@ -1270,10 +1196,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.0017578125</v>
+        <v>0.00078125</v>
       </c>
       <c r="C36" t="n">
-        <v>0.001953125</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="37">
@@ -1283,10 +1209,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.0037109375</v>
+        <v>0.00234375</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0013671875</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="38">
@@ -1296,10 +1222,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.0015625</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C38" t="n">
-        <v>0.003125</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="39">
@@ -1309,10 +1235,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.0025390625</v>
+        <v>0.0029296875</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0025390625</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="40">
@@ -1322,10 +1248,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.00234375</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C40" t="n">
-        <v>0.0029296875</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="41">
@@ -1335,10 +1261,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.003515625</v>
+        <v>0.0015625</v>
       </c>
       <c r="C41" t="n">
-        <v>0.004296875</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="42">
@@ -1348,10 +1274,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.00234375</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0015625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="43">
@@ -1361,10 +1287,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.004296875</v>
+        <v>0.01015625</v>
       </c>
       <c r="C43" t="n">
-        <v>0.00078125</v>
+        <v>0.00546875</v>
       </c>
     </row>
     <row r="44">
@@ -1374,10 +1300,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.0017578125</v>
+        <v>0.0001953125</v>
       </c>
       <c r="C44" t="n">
-        <v>0.001953125</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="45">
@@ -1390,7 +1316,7 @@
         <v>0.00078125</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0009765625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="46">
@@ -1400,7 +1326,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.005859375</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C46" t="n">
         <v>0.0013671875</v>
@@ -1413,10 +1339,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.00546875</v>
+        <v>0.0021484375</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0021484375</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="48">
@@ -1426,10 +1352,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.0017578125</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C48" t="n">
-        <v>0.001953125</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="49">
@@ -1439,10 +1365,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.0025390625</v>
+        <v>0.0015625</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0029296875</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="50">
@@ -1452,10 +1378,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.0046875</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C50" t="n">
-        <v>0.005078125</v>
+        <v>0.0056640625</v>
       </c>
     </row>
     <row r="51">
@@ -1465,10 +1391,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.006640625</v>
+        <v>0.01796875</v>
       </c>
       <c r="C51" t="n">
-        <v>0.008593750000000001</v>
+        <v>0.0111328125</v>
       </c>
     </row>
     <row r="52">
@@ -1478,10 +1404,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.003125</v>
+        <v>0.0015625</v>
       </c>
       <c r="C52" t="n">
-        <v>0.00546875</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="53">
@@ -1491,10 +1417,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.007421875</v>
+        <v>0.005859375</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0078125</v>
+        <v>0.009375</v>
       </c>
     </row>
     <row r="54">
@@ -1504,10 +1430,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.005078125</v>
+        <v>0.0033203125</v>
       </c>
       <c r="C54" t="n">
-        <v>0.002734375</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="55">
@@ -1517,10 +1443,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.003125</v>
+        <v>0.008984374999999999</v>
       </c>
       <c r="C55" t="n">
-        <v>0.0017578125</v>
+        <v>0.00390625</v>
       </c>
     </row>
     <row r="56">
@@ -1530,10 +1456,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.0056640625</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C56" t="n">
-        <v>0.0021484375</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="57">
@@ -1543,10 +1469,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.00625</v>
+        <v>0.0015625</v>
       </c>
       <c r="C57" t="n">
-        <v>0.0013671875</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="58">
@@ -1556,10 +1482,10 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.005859375</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C58" t="n">
-        <v>0.0041015625</v>
+        <v>0.00703125</v>
       </c>
     </row>
     <row r="59">
@@ -1569,10 +1495,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.0091796875</v>
+        <v>0.016015625</v>
       </c>
       <c r="C59" t="n">
-        <v>0.00390625</v>
+        <v>0.01875</v>
       </c>
     </row>
     <row r="60">
@@ -1582,10 +1508,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.003125</v>
+        <v>0.00234375</v>
       </c>
       <c r="C60" t="n">
-        <v>0.005859375</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="61">
@@ -1595,10 +1521,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.00703125</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C61" t="n">
-        <v>0.01015625</v>
+        <v>0.006640625</v>
       </c>
     </row>
     <row r="62">
@@ -1608,10 +1534,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.006640625</v>
+        <v>0.0044921875</v>
       </c>
       <c r="C62" t="n">
-        <v>0.003125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="63">
@@ -1621,10 +1547,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.009375</v>
+        <v>0.0091796875</v>
       </c>
       <c r="C63" t="n">
-        <v>0.0029296875</v>
+        <v>0.0068359375</v>
       </c>
     </row>
     <row r="64">
@@ -1634,10 +1560,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.0033203125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C64" t="n">
-        <v>0.002734375</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="65">
@@ -1647,10 +1573,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.003515625</v>
+        <v>0.003125</v>
       </c>
       <c r="C65" t="n">
-        <v>0.0046875</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="66">
@@ -1660,7 +1586,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.00078125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C66" t="n">
         <v>0.0017578125</v>
@@ -1673,10 +1599,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.002734375</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C67" t="n">
-        <v>0.0048828125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="68">
@@ -1686,10 +1612,10 @@
         </is>
       </c>
       <c r="B68" t="n">
+        <v>0.0056640625</v>
+      </c>
+      <c r="C68" t="n">
         <v>0.001953125</v>
-      </c>
-      <c r="C68" t="n">
-        <v>0.0021484375</v>
       </c>
     </row>
     <row r="69">
@@ -1699,10 +1625,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.0041015625</v>
+        <v>0.0060546875</v>
       </c>
       <c r="C69" t="n">
-        <v>0.00546875</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="70">
@@ -1712,10 +1638,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.0009765625</v>
+        <v>0.00234375</v>
       </c>
       <c r="C70" t="n">
-        <v>0.0025390625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="71">
@@ -1725,10 +1651,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.002734375</v>
+        <v>0.003125</v>
       </c>
       <c r="C71" t="n">
-        <v>0.0078125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="72">
@@ -1738,10 +1664,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.003125</v>
+        <v>0.009375</v>
       </c>
       <c r="C72" t="n">
-        <v>0.0052734375</v>
+        <v>0.004296875</v>
       </c>
     </row>
     <row r="73">
@@ -1751,10 +1677,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.0076171875</v>
+        <v>0.0044921875</v>
       </c>
       <c r="C73" t="n">
-        <v>0.0138671875</v>
+        <v>0.00546875</v>
       </c>
     </row>
     <row r="74">
@@ -1764,7 +1690,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.00078125</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C74" t="n">
         <v>0.0015625</v>
@@ -1777,10 +1703,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.0048828125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C75" t="n">
-        <v>0.0048828125</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="76">
@@ -1790,10 +1716,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.0009765625</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C76" t="n">
-        <v>0.0017578125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="77">
@@ -1803,10 +1729,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.0041015625</v>
+        <v>0.00703125</v>
       </c>
       <c r="C77" t="n">
-        <v>0.00625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="78">
@@ -1816,10 +1742,10 @@
         </is>
       </c>
       <c r="B78" t="n">
+        <v>0.0017578125</v>
+      </c>
+      <c r="C78" t="n">
         <v>0.00234375</v>
-      </c>
-      <c r="C78" t="n">
-        <v>0.0060546875</v>
       </c>
     </row>
     <row r="79">
@@ -1829,10 +1755,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.00546875</v>
+        <v>0.002734375</v>
       </c>
       <c r="C79" t="n">
-        <v>0.01015625</v>
+        <v>0.01796875</v>
       </c>
     </row>
     <row r="80">
@@ -1842,10 +1768,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.0015625</v>
+        <v>0.005859375</v>
       </c>
       <c r="C80" t="n">
-        <v>0.0037109375</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="81">
@@ -1855,10 +1781,10 @@
         </is>
       </c>
       <c r="B81" t="n">
+        <v>0.0068359375</v>
+      </c>
+      <c r="C81" t="n">
         <v>0.00703125</v>
-      </c>
-      <c r="C81" t="n">
-        <v>0.007421875</v>
       </c>
     </row>
     <row r="82">
@@ -1868,10 +1794,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.0013671875</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C82" t="n">
-        <v>0.0021484375</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="83">
@@ -1881,7 +1807,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.003125</v>
+        <v>0.001953125</v>
       </c>
       <c r="C83" t="n">
         <v>0.0029296875</v>
@@ -1894,10 +1820,10 @@
         </is>
       </c>
       <c r="B84" t="n">
+        <v>0.003515625</v>
+      </c>
+      <c r="C84" t="n">
         <v>0.0044921875</v>
-      </c>
-      <c r="C84" t="n">
-        <v>0.003125</v>
       </c>
     </row>
     <row r="85">
@@ -1907,10 +1833,10 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.0142578125</v>
+        <v>0.0107421875</v>
       </c>
       <c r="C85" t="n">
-        <v>0.0048828125</v>
+        <v>0.005078125</v>
       </c>
     </row>
     <row r="86">
@@ -1920,10 +1846,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.001171875</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C86" t="n">
-        <v>0.0015625</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="87">
@@ -1933,10 +1859,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.0021484375</v>
+        <v>0.00234375</v>
       </c>
       <c r="C87" t="n">
-        <v>0.0044921875</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="88">
@@ -1946,10 +1872,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.0029296875</v>
+        <v>0.005859375</v>
       </c>
       <c r="C88" t="n">
-        <v>0.00234375</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="89">
@@ -1959,10 +1885,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.008593750000000001</v>
+        <v>0.008984374999999999</v>
       </c>
       <c r="C89" t="n">
-        <v>0.008007812499999999</v>
+        <v>0.004296875</v>
       </c>
     </row>
     <row r="90">
@@ -1972,10 +1898,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.0029296875</v>
+        <v>0</v>
       </c>
       <c r="C90" t="n">
-        <v>0.00390625</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="91">
@@ -1985,10 +1911,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.00546875</v>
+        <v>0.0015625</v>
       </c>
       <c r="C91" t="n">
-        <v>0.0037109375</v>
+        <v>0.00390625</v>
       </c>
     </row>
     <row r="92">
@@ -1998,10 +1924,10 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.0025390625</v>
+        <v>0.001953125</v>
       </c>
       <c r="C92" t="n">
-        <v>0.00234375</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="93">
@@ -2011,10 +1937,10 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.00546875</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C93" t="n">
-        <v>0.00234375</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="94">
@@ -2024,7 +1950,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.0017578125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C94" t="n">
         <v>0.0025390625</v>
@@ -2037,10 +1963,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.0033203125</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C95" t="n">
-        <v>0.00390625</v>
+        <v>0.0140625</v>
       </c>
     </row>
     <row r="96">
@@ -2050,10 +1976,10 @@
         </is>
       </c>
       <c r="B96" t="n">
+        <v>0.0029296875</v>
+      </c>
+      <c r="C96" t="n">
         <v>0.0015625</v>
-      </c>
-      <c r="C96" t="n">
-        <v>0.0021484375</v>
       </c>
     </row>
     <row r="97">
@@ -2063,10 +1989,10 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.0025390625</v>
+        <v>0.003515625</v>
       </c>
       <c r="C97" t="n">
-        <v>0.004296875</v>
+        <v>0.0076171875</v>
       </c>
     </row>
     <row r="98">
@@ -2076,10 +2002,10 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.000390625</v>
+        <v>0.0033203125</v>
       </c>
       <c r="C98" t="n">
-        <v>0.003125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="99">
@@ -2089,10 +2015,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.0041015625</v>
+        <v>0.005859375</v>
       </c>
       <c r="C99" t="n">
-        <v>0.0046875</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="100">
@@ -2102,10 +2028,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.000390625</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0021484375</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="101">
@@ -2115,10 +2041,10 @@
         </is>
       </c>
       <c r="B101" t="n">
+        <v>0.0017578125</v>
+      </c>
+      <c r="C101" t="n">
         <v>0.0029296875</v>
-      </c>
-      <c r="C101" t="n">
-        <v>0.0044921875</v>
       </c>
     </row>
     <row r="102">
@@ -2128,7 +2054,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.0013671875</v>
+        <v>0.008007812499999999</v>
       </c>
       <c r="C102" t="n">
         <v>0.0025390625</v>
@@ -2141,10 +2067,10 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.005859375</v>
+        <v>0.006640625</v>
       </c>
       <c r="C103" t="n">
-        <v>0.008007812499999999</v>
+        <v>0.00703125</v>
       </c>
     </row>
     <row r="104">
@@ -2154,10 +2080,10 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.0015625</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C104" t="n">
-        <v>0.0046875</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="105">
@@ -2167,10 +2093,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.00625</v>
+        <v>0.001171875</v>
       </c>
       <c r="C105" t="n">
-        <v>0.008984374999999999</v>
+        <v>0.0166015625</v>
       </c>
     </row>
     <row r="106">
@@ -2180,10 +2106,10 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.0029296875</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C106" t="n">
-        <v>0.0025390625</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="107">
@@ -2193,10 +2119,10 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.00546875</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C107" t="n">
-        <v>0.007421875</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="108">
@@ -2206,10 +2132,10 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0</v>
+        <v>0.001171875</v>
       </c>
       <c r="C108" t="n">
-        <v>0.0029296875</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="109">
@@ -2219,10 +2145,10 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.0015625</v>
+        <v>0.002734375</v>
       </c>
       <c r="C109" t="n">
-        <v>0.0056640625</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="110">
@@ -2232,10 +2158,10 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.0025390625</v>
+        <v>0.008007812499999999</v>
       </c>
       <c r="C110" t="n">
-        <v>0.0029296875</v>
+        <v>0.00546875</v>
       </c>
     </row>
     <row r="111">
@@ -2245,10 +2171,10 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.008203125</v>
+        <v>0.002734375</v>
       </c>
       <c r="C111" t="n">
-        <v>0.0111328125</v>
+        <v>0.00546875</v>
       </c>
     </row>
     <row r="112">
@@ -2258,10 +2184,10 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.00078125</v>
+        <v>0.00234375</v>
       </c>
       <c r="C112" t="n">
-        <v>0.0041015625</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="113">
@@ -2271,10 +2197,10 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.0029296875</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C113" t="n">
-        <v>0.008203125</v>
+        <v>0.003515625</v>
       </c>
     </row>
     <row r="114">
@@ -2284,10 +2210,10 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.0041015625</v>
+        <v>0.001953125</v>
       </c>
       <c r="C114" t="n">
-        <v>0.001953125</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="115">
@@ -2297,10 +2223,10 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.002734375</v>
+        <v>0.004296875</v>
       </c>
       <c r="C115" t="n">
-        <v>0.003515625</v>
+        <v>0.0041015625</v>
       </c>
     </row>
     <row r="116">
@@ -2310,10 +2236,10 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.00234375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C116" t="n">
-        <v>0.00390625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="117">
@@ -2323,10 +2249,10 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.0060546875</v>
+        <v>0.0015625</v>
       </c>
       <c r="C117" t="n">
-        <v>0.0025390625</v>
+        <v>0.00390625</v>
       </c>
     </row>
     <row r="118">
@@ -2336,10 +2262,10 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.0021484375</v>
+        <v>0.003515625</v>
       </c>
       <c r="C118" t="n">
-        <v>0.003515625</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="119">
@@ -2349,10 +2275,10 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.00390625</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C119" t="n">
-        <v>0.0046875</v>
+        <v>0.00703125</v>
       </c>
     </row>
     <row r="120">
@@ -2362,10 +2288,10 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.0025390625</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C120" t="n">
-        <v>0.0025390625</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="121">
@@ -2375,10 +2301,10 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.005859375</v>
+        <v>0.00078125</v>
       </c>
       <c r="C121" t="n">
-        <v>0.005859375</v>
+        <v>0.013671875</v>
       </c>
     </row>
     <row r="122">
@@ -2388,7 +2314,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.00390625</v>
+        <v>0.0033203125</v>
       </c>
       <c r="C122" t="n">
         <v>0.002734375</v>
@@ -2401,10 +2327,10 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.0125</v>
+        <v>0.007421875</v>
       </c>
       <c r="C123" t="n">
-        <v>0.0046875</v>
+        <v>0.00546875</v>
       </c>
     </row>
     <row r="124">
@@ -2414,10 +2340,10 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.00078125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C124" t="n">
-        <v>0.003125</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="125">
@@ -2427,10 +2353,10 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.002734375</v>
+        <v>0.00078125</v>
       </c>
       <c r="C125" t="n">
-        <v>0.0037109375</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="126">
@@ -2440,7 +2366,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.003515625</v>
+        <v>0.0056640625</v>
       </c>
       <c r="C126" t="n">
         <v>0.0021484375</v>
@@ -2453,10 +2379,10 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.007421875</v>
+        <v>0.0103515625</v>
       </c>
       <c r="C127" t="n">
-        <v>0.0119140625</v>
+        <v>0.0056640625</v>
       </c>
     </row>
     <row r="128">
@@ -2466,10 +2392,10 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.0013671875</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C128" t="n">
-        <v>0.0025390625</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="129">
@@ -2479,10 +2405,10 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.0017578125</v>
+        <v>0.0015625</v>
       </c>
       <c r="C129" t="n">
-        <v>0.0046875</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="130">
@@ -2492,10 +2418,10 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.0029296875</v>
+        <v>0.0021484375</v>
       </c>
       <c r="C130" t="n">
-        <v>0.0046875</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="131">
@@ -2505,10 +2431,10 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.0015625</v>
+        <v>0.001171875</v>
       </c>
       <c r="C131" t="n">
-        <v>0.0021484375</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="132">
@@ -2518,10 +2444,10 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.01015625</v>
+        <v>0.008984374999999999</v>
       </c>
       <c r="C132" t="n">
-        <v>0.008007812499999999</v>
+        <v>0.0044921875</v>
       </c>
     </row>
     <row r="133">
@@ -2531,10 +2457,10 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.002734375</v>
+        <v>0.0068359375</v>
       </c>
       <c r="C133" t="n">
-        <v>0.0017578125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="134">
@@ -2544,10 +2470,10 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.0025390625</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C134" t="n">
-        <v>0.0048828125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="135">
@@ -2557,10 +2483,10 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.0013671875</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C135" t="n">
-        <v>0.0064453125</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="136">
@@ -2570,10 +2496,10 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.0111328125</v>
+        <v>0.009570312500000001</v>
       </c>
       <c r="C136" t="n">
-        <v>0.00546875</v>
+        <v>0.0072265625</v>
       </c>
     </row>
     <row r="137">
@@ -2583,10 +2509,10 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.00390625</v>
+        <v>0.0021484375</v>
       </c>
       <c r="C137" t="n">
-        <v>0.0033203125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="138">
@@ -2596,10 +2522,10 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.0044921875</v>
+        <v>0.00234375</v>
       </c>
       <c r="C138" t="n">
-        <v>0.0048828125</v>
+        <v>0.0140625</v>
       </c>
     </row>
     <row r="139">
@@ -2609,10 +2535,10 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.0021484375</v>
+        <v>0.0015625</v>
       </c>
       <c r="C139" t="n">
-        <v>0.001953125</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="140">
@@ -2622,10 +2548,10 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>0.0025390625</v>
+        <v>0.003125</v>
       </c>
       <c r="C140" t="n">
-        <v>0.0056640625</v>
+        <v>0.0078125</v>
       </c>
     </row>
     <row r="141">
@@ -2635,10 +2561,10 @@
         </is>
       </c>
       <c r="B141" t="n">
+        <v>0.0037109375</v>
+      </c>
+      <c r="C141" t="n">
         <v>0.001953125</v>
-      </c>
-      <c r="C141" t="n">
-        <v>0.002734375</v>
       </c>
     </row>
     <row r="142">
@@ -2648,10 +2574,10 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.00625</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C142" t="n">
-        <v>0.002734375</v>
+        <v>0.0048828125</v>
       </c>
     </row>
     <row r="143">
@@ -2661,10 +2587,10 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.0015625</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C143" t="n">
-        <v>0.0048828125</v>
+        <v>0.0009765625</v>
       </c>
     </row>
     <row r="144">
@@ -2674,10 +2600,10 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>0.0029296875</v>
+        <v>0.00546875</v>
       </c>
       <c r="C144" t="n">
-        <v>0.0025390625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="145">
@@ -2687,10 +2613,10 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.001953125</v>
+        <v>0.00234375</v>
       </c>
       <c r="C145" t="n">
-        <v>0.0021484375</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="146">
@@ -2700,10 +2626,10 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>0.0033203125</v>
+        <v>0.00234375</v>
       </c>
       <c r="C146" t="n">
-        <v>0.006640625</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="147">
@@ -2713,10 +2639,10 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.00078125</v>
+        <v>0.0029296875</v>
       </c>
       <c r="C147" t="n">
-        <v>0.0037109375</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="148">
@@ -2726,10 +2652,10 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.0083984375</v>
+        <v>0.00546875</v>
       </c>
       <c r="C148" t="n">
-        <v>0.0115234375</v>
+        <v>0.0068359375</v>
       </c>
     </row>
     <row r="149">
@@ -2739,10 +2665,10 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0.00234375</v>
+        <v>0.008984374999999999</v>
       </c>
       <c r="C149" t="n">
-        <v>0.0048828125</v>
+        <v>0.0041015625</v>
       </c>
     </row>
     <row r="150">
@@ -2752,10 +2678,10 @@
         </is>
       </c>
       <c r="B150" t="n">
+        <v>0.0017578125</v>
+      </c>
+      <c r="C150" t="n">
         <v>0.0029296875</v>
-      </c>
-      <c r="C150" t="n">
-        <v>0.0056640625</v>
       </c>
     </row>
     <row r="151">
@@ -2765,10 +2691,10 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.0001953125</v>
+        <v>0.0015625</v>
       </c>
       <c r="C151" t="n">
-        <v>0.001171875</v>
+        <v>0.00078125</v>
       </c>
     </row>
     <row r="152">
@@ -2778,10 +2704,10 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>0.0044921875</v>
+        <v>0.0048828125</v>
       </c>
       <c r="C152" t="n">
-        <v>0.0068359375</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="153">
@@ -2791,10 +2717,10 @@
         </is>
       </c>
       <c r="B153" t="n">
+        <v>0.00546875</v>
+      </c>
+      <c r="C153" t="n">
         <v>0.0017578125</v>
-      </c>
-      <c r="C153" t="n">
-        <v>0.001171875</v>
       </c>
     </row>
     <row r="154">
@@ -2804,10 +2730,10 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.00625</v>
+        <v>0.001953125</v>
       </c>
       <c r="C154" t="n">
-        <v>0.009375</v>
+        <v>0.0142578125</v>
       </c>
     </row>
     <row r="155">
@@ -2817,10 +2743,10 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.0015625</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C155" t="n">
-        <v>0.0041015625</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="156">
@@ -2830,10 +2756,10 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>0.0060546875</v>
+        <v>0.0064453125</v>
       </c>
       <c r="C156" t="n">
-        <v>0.005078125</v>
+        <v>0.0072265625</v>
       </c>
     </row>
     <row r="157">
@@ -2843,10 +2769,10 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>0.002734375</v>
+        <v>0.0068359375</v>
       </c>
       <c r="C157" t="n">
-        <v>0.003515625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="158">
@@ -2856,10 +2782,10 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.0044921875</v>
+        <v>0.001171875</v>
       </c>
       <c r="C158" t="n">
-        <v>0.00546875</v>
+        <v>0.00390625</v>
       </c>
     </row>
     <row r="159">
@@ -2869,10 +2795,10 @@
         </is>
       </c>
       <c r="B159" t="n">
+        <v>0.000390625</v>
+      </c>
+      <c r="C159" t="n">
         <v>0.0013671875</v>
-      </c>
-      <c r="C159" t="n">
-        <v>0.003515625</v>
       </c>
     </row>
     <row r="160">
@@ -2882,10 +2808,10 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>0.0041015625</v>
+        <v>0.00625</v>
       </c>
       <c r="C160" t="n">
-        <v>0.00390625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="161">
@@ -2895,10 +2821,10 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.0005859375</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C161" t="n">
-        <v>0.0021484375</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="162">
@@ -2908,10 +2834,10 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.004296875</v>
+        <v>0.00546875</v>
       </c>
       <c r="C162" t="n">
-        <v>0.0056640625</v>
+        <v>0.008593750000000001</v>
       </c>
     </row>
     <row r="163">
@@ -2921,10 +2847,10 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.0015625</v>
+        <v>0.0046875</v>
       </c>
       <c r="C163" t="n">
-        <v>0.002734375</v>
+        <v>0.000390625</v>
       </c>
     </row>
     <row r="164">
@@ -2934,10 +2860,10 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.00625</v>
+        <v>0.001953125</v>
       </c>
       <c r="C164" t="n">
-        <v>0.0044921875</v>
+        <v>0.0115234375</v>
       </c>
     </row>
     <row r="165">
@@ -2947,10 +2873,10 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.001953125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C165" t="n">
-        <v>0.003125</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="166">
@@ -2960,10 +2886,10 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>0.005078125</v>
+        <v>0.003125</v>
       </c>
       <c r="C166" t="n">
-        <v>0.004296875</v>
+        <v>0.003515625</v>
       </c>
     </row>
     <row r="167">
@@ -2973,10 +2899,10 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.0025390625</v>
+        <v>0.0033203125</v>
       </c>
       <c r="C167" t="n">
-        <v>0.00234375</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="168">
@@ -2986,10 +2912,10 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.00546875</v>
+        <v>0.00234375</v>
       </c>
       <c r="C168" t="n">
-        <v>0.0025390625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="169">
@@ -2999,10 +2925,10 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.0017578125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C169" t="n">
-        <v>0.00390625</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="170">
@@ -3012,10 +2938,10 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>0.007421875</v>
+        <v>0.009765625</v>
       </c>
       <c r="C170" t="n">
-        <v>0.0076171875</v>
+        <v>0.004296875</v>
       </c>
     </row>
     <row r="171">
@@ -3025,10 +2951,10 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.002734375</v>
+        <v>0.0064453125</v>
       </c>
       <c r="C171" t="n">
-        <v>0.004296875</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="172">
@@ -3038,10 +2964,10 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.0029296875</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C172" t="n">
-        <v>0.0044921875</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="173">
@@ -3051,10 +2977,10 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.000390625</v>
+        <v>0.00078125</v>
       </c>
       <c r="C173" t="n">
-        <v>0.0033203125</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="174">
@@ -3064,10 +2990,10 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>0.0142578125</v>
+        <v>0.0091796875</v>
       </c>
       <c r="C174" t="n">
-        <v>0.0025390625</v>
+        <v>0.0044921875</v>
       </c>
     </row>
     <row r="175">
@@ -3077,10 +3003,10 @@
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0.0064453125</v>
+        <v>0.0029296875</v>
       </c>
       <c r="C175" t="n">
-        <v>0.0025390625</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="176">
@@ -3090,10 +3016,10 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>0.0033203125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C176" t="n">
-        <v>0.00234375</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="177">
@@ -3103,10 +3029,10 @@
         </is>
       </c>
       <c r="B177" t="n">
+        <v>0.0005859375</v>
+      </c>
+      <c r="C177" t="n">
         <v>0.0013671875</v>
-      </c>
-      <c r="C177" t="n">
-        <v>0.0029296875</v>
       </c>
     </row>
     <row r="178">
@@ -3116,10 +3042,10 @@
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.0048828125</v>
+        <v>0.00625</v>
       </c>
       <c r="C178" t="n">
-        <v>0.0060546875</v>
+        <v>0.009765625</v>
       </c>
     </row>
     <row r="179">
@@ -3129,10 +3055,10 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.0025390625</v>
+        <v>0.00625</v>
       </c>
       <c r="C179" t="n">
-        <v>0.003125</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="180">
@@ -3142,10 +3068,10 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.0078125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C180" t="n">
-        <v>0.008203125</v>
+        <v>0.0169921875</v>
       </c>
     </row>
     <row r="181">
@@ -3155,10 +3081,10 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.0015625</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C181" t="n">
-        <v>0.003125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="182">
@@ -3168,10 +3094,10 @@
         </is>
       </c>
       <c r="B182" t="n">
-        <v>0.0056640625</v>
+        <v>0.0044921875</v>
       </c>
       <c r="C182" t="n">
-        <v>0.0041015625</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="183">
@@ -3181,10 +3107,10 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.0009765625</v>
+        <v>0.005078125</v>
       </c>
       <c r="C183" t="n">
-        <v>0.001953125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="184">
@@ -3194,10 +3120,10 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.005859375</v>
+        <v>0.0021484375</v>
       </c>
       <c r="C184" t="n">
-        <v>0.0052734375</v>
+        <v>0.0046875</v>
       </c>
     </row>
     <row r="185">
@@ -3207,10 +3133,10 @@
         </is>
       </c>
       <c r="B185" t="n">
+        <v>0.0013671875</v>
+      </c>
+      <c r="C185" t="n">
         <v>0.001171875</v>
-      </c>
-      <c r="C185" t="n">
-        <v>0.0029296875</v>
       </c>
     </row>
     <row r="186">
@@ -3220,10 +3146,10 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0.00703125</v>
+        <v>0.0046875</v>
       </c>
       <c r="C186" t="n">
-        <v>0.0138671875</v>
+        <v>0.0076171875</v>
       </c>
     </row>
     <row r="187">
@@ -3233,7 +3159,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0.0029296875</v>
+        <v>0.008593750000000001</v>
       </c>
       <c r="C187" t="n">
         <v>0.005078125</v>
@@ -3246,10 +3172,10 @@
         </is>
       </c>
       <c r="B188" t="n">
-        <v>0.002734375</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C188" t="n">
-        <v>0.009765625</v>
+        <v>0.00390625</v>
       </c>
     </row>
     <row r="189">
@@ -3259,10 +3185,10 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.000390625</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C189" t="n">
-        <v>0.0033203125</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="190">
@@ -3272,10 +3198,10 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0.0060546875</v>
+        <v>0.00703125</v>
       </c>
       <c r="C190" t="n">
-        <v>0.005859375</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="191">
@@ -3285,10 +3211,10 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.001171875</v>
+        <v>0.007421875</v>
       </c>
       <c r="C191" t="n">
-        <v>0.0021484375</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="192">
@@ -3298,10 +3224,10 @@
         </is>
       </c>
       <c r="B192" t="n">
+        <v>0.001171875</v>
+      </c>
+      <c r="C192" t="n">
         <v>0.002734375</v>
-      </c>
-      <c r="C192" t="n">
-        <v>0.004296875</v>
       </c>
     </row>
     <row r="193">
@@ -3311,10 +3237,10 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>0.000390625</v>
+        <v>0.00078125</v>
       </c>
       <c r="C193" t="n">
-        <v>0.0025390625</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="194">
@@ -3324,10 +3250,10 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.003515625</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C194" t="n">
-        <v>0.00234375</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="195">
@@ -3337,10 +3263,10 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.0037109375</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C195" t="n">
-        <v>0.00390625</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="196">
@@ -3350,10 +3276,10 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>0.0072265625</v>
+        <v>0.01015625</v>
       </c>
       <c r="C196" t="n">
-        <v>0.003125</v>
+        <v>0.0041015625</v>
       </c>
     </row>
     <row r="197">
@@ -3363,10 +3289,10 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>0.0044921875</v>
+        <v>0.0029296875</v>
       </c>
       <c r="C197" t="n">
-        <v>0.0025390625</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="198">
@@ -3376,10 +3302,10 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>0.0044921875</v>
+        <v>0.00546875</v>
       </c>
       <c r="C198" t="n">
-        <v>0.0125</v>
+        <v>0.0064453125</v>
       </c>
     </row>
     <row r="199">
@@ -3389,10 +3315,10 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>0.001953125</v>
+        <v>0.0025390625</v>
       </c>
       <c r="C199" t="n">
-        <v>0.0072265625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="200">
@@ -3402,10 +3328,10 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>0.0134765625</v>
+        <v>0.0185546875</v>
       </c>
       <c r="C200" t="n">
-        <v>0.005859375</v>
+        <v>0.0158203125</v>
       </c>
     </row>
     <row r="201">
@@ -3415,10 +3341,10 @@
         </is>
       </c>
       <c r="B201" t="n">
-        <v>0.0041015625</v>
+        <v>0.005078125</v>
       </c>
       <c r="C201" t="n">
-        <v>0.004296875</v>
+        <v>0.008007812499999999</v>
       </c>
     </row>
     <row r="202">
@@ -3428,10 +3354,10 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>0.005078125</v>
+        <v>0.002734375</v>
       </c>
       <c r="C202" t="n">
-        <v>0.001953125</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="203">
@@ -3441,10 +3367,10 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>0.004296875</v>
+        <v>0.000390625</v>
       </c>
       <c r="C203" t="n">
-        <v>0.005078125</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="204">
@@ -3454,10 +3380,10 @@
         </is>
       </c>
       <c r="B204" t="n">
-        <v>0.0037109375</v>
+        <v>0.009375</v>
       </c>
       <c r="C204" t="n">
-        <v>0.0033203125</v>
+        <v>0.005078125</v>
       </c>
     </row>
     <row r="205">
@@ -3467,10 +3393,10 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>0.00546875</v>
+        <v>0.003125</v>
       </c>
       <c r="C205" t="n">
-        <v>0.0025390625</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="206">
@@ -3480,10 +3406,10 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>0.009960937499999999</v>
+        <v>0.00390625</v>
       </c>
       <c r="C206" t="n">
-        <v>0.00546875</v>
+        <v>0.009375</v>
       </c>
     </row>
     <row r="207">
@@ -3493,10 +3419,10 @@
         </is>
       </c>
       <c r="B207" t="n">
-        <v>0.0052734375</v>
+        <v>0.00390625</v>
       </c>
       <c r="C207" t="n">
-        <v>0.005078125</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="208">
@@ -3506,10 +3432,10 @@
         </is>
       </c>
       <c r="B208" t="n">
-        <v>0.0068359375</v>
+        <v>0.0193359375</v>
       </c>
       <c r="C208" t="n">
-        <v>0.0064453125</v>
+        <v>0.011328125</v>
       </c>
     </row>
     <row r="209">
@@ -3519,10 +3445,10 @@
         </is>
       </c>
       <c r="B209" t="n">
-        <v>0.004296875</v>
+        <v>0.0052734375</v>
       </c>
       <c r="C209" t="n">
-        <v>0.00703125</v>
+        <v>0.0052734375</v>
       </c>
     </row>
     <row r="210">
@@ -3532,10 +3458,10 @@
         </is>
       </c>
       <c r="B210" t="n">
-        <v>0.0021484375</v>
+        <v>0.000390625</v>
       </c>
       <c r="C210" t="n">
-        <v>0.0033203125</v>
+        <v>0.0025390625</v>
       </c>
     </row>
     <row r="211">
@@ -3545,10 +3471,10 @@
         </is>
       </c>
       <c r="B211" t="n">
-        <v>0.001953125</v>
+        <v>0.00078125</v>
       </c>
       <c r="C211" t="n">
-        <v>0.0025390625</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="212">
@@ -3558,10 +3484,10 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>0.0060546875</v>
+        <v>0.001953125</v>
       </c>
       <c r="C212" t="n">
-        <v>0.003125</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="213">
@@ -3571,10 +3497,10 @@
         </is>
       </c>
       <c r="B213" t="n">
-        <v>0.004296875</v>
+        <v>0.0044921875</v>
       </c>
       <c r="C213" t="n">
-        <v>0.0009765625</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="214">
@@ -3584,10 +3510,10 @@
         </is>
       </c>
       <c r="B214" t="n">
-        <v>0.0009765625</v>
+        <v>0.001171875</v>
       </c>
       <c r="C214" t="n">
-        <v>0.0009765625</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="215">
@@ -3597,10 +3523,10 @@
         </is>
       </c>
       <c r="B215" t="n">
-        <v>0.001171875</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C215" t="n">
-        <v>0.0013671875</v>
+        <v>0.0015625</v>
       </c>
     </row>
     <row r="216">
@@ -3610,10 +3536,10 @@
         </is>
       </c>
       <c r="B216" t="n">
-        <v>0.0060546875</v>
+        <v>0.009765625</v>
       </c>
       <c r="C216" t="n">
-        <v>0.0013671875</v>
+        <v>0.005859375</v>
       </c>
     </row>
     <row r="217">
@@ -3623,10 +3549,10 @@
         </is>
       </c>
       <c r="B217" t="n">
+        <v>0.00390625</v>
+      </c>
+      <c r="C217" t="n">
         <v>0.0029296875</v>
-      </c>
-      <c r="C217" t="n">
-        <v>0.000390625</v>
       </c>
     </row>
     <row r="218">
@@ -3636,10 +3562,10 @@
         </is>
       </c>
       <c r="B218" t="n">
-        <v>0.0046875</v>
+        <v>0.0021484375</v>
       </c>
       <c r="C218" t="n">
-        <v>0.00390625</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="219">
@@ -3649,10 +3575,10 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>0.002734375</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C219" t="n">
-        <v>0.0009765625</v>
+        <v>0.001171875</v>
       </c>
     </row>
     <row r="220">
@@ -3662,10 +3588,10 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>0.003125</v>
+        <v>0.002734375</v>
       </c>
       <c r="C220" t="n">
-        <v>0.00390625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="221">
@@ -3675,10 +3601,10 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>0.001953125</v>
+        <v>0.002734375</v>
       </c>
       <c r="C221" t="n">
-        <v>0.0025390625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="222">
@@ -3688,10 +3614,10 @@
         </is>
       </c>
       <c r="B222" t="n">
-        <v>0.002734375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C222" t="n">
-        <v>0.0013671875</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="223">
@@ -3701,10 +3627,10 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>0.001953125</v>
+        <v>0.00078125</v>
       </c>
       <c r="C223" t="n">
-        <v>0.0009765625</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="224">
@@ -3714,10 +3640,10 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>0.001171875</v>
+        <v>0.00703125</v>
       </c>
       <c r="C224" t="n">
-        <v>0.001171875</v>
+        <v>0.0044921875</v>
       </c>
     </row>
     <row r="225">
@@ -3727,10 +3653,10 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>0.003125</v>
+        <v>0.0017578125</v>
       </c>
       <c r="C225" t="n">
-        <v>0.001171875</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="226">
@@ -3740,10 +3666,10 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>0.006640625</v>
+        <v>0.008593750000000001</v>
       </c>
       <c r="C226" t="n">
-        <v>0.001953125</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="227">
@@ -3753,10 +3679,10 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>0.00625</v>
+        <v>0.0015625</v>
       </c>
       <c r="C227" t="n">
-        <v>0.0017578125</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="228">
@@ -3766,10 +3692,10 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>0.00625</v>
+        <v>0.00234375</v>
       </c>
       <c r="C228" t="n">
-        <v>0.001953125</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="229">
@@ -3779,10 +3705,10 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>0.005078125</v>
+        <v>0.001171875</v>
       </c>
       <c r="C229" t="n">
-        <v>0.0017578125</v>
+        <v>0.0013671875</v>
       </c>
     </row>
     <row r="230">
@@ -3792,10 +3718,10 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>0.0060546875</v>
+        <v>0.023046875</v>
       </c>
       <c r="C230" t="n">
-        <v>0.0083984375</v>
+        <v>0.0125</v>
       </c>
     </row>
     <row r="231">
@@ -3805,10 +3731,10 @@
         </is>
       </c>
       <c r="B231" t="n">
-        <v>0.0037109375</v>
+        <v>0.0044921875</v>
       </c>
       <c r="C231" t="n">
-        <v>0.0087890625</v>
+        <v>0.0046875</v>
       </c>
     </row>
     <row r="232">
@@ -3818,10 +3744,10 @@
         </is>
       </c>
       <c r="B232" t="n">
-        <v>0.0083984375</v>
+        <v>0.0041015625</v>
       </c>
       <c r="C232" t="n">
-        <v>0.00546875</v>
+        <v>0.009375</v>
       </c>
     </row>
     <row r="233">
@@ -3831,10 +3757,10 @@
         </is>
       </c>
       <c r="B233" t="n">
-        <v>0.0037109375</v>
+        <v>0.00234375</v>
       </c>
       <c r="C233" t="n">
-        <v>0.0064453125</v>
+        <v>0.0044921875</v>
       </c>
     </row>
     <row r="234">
@@ -3844,10 +3770,10 @@
         </is>
       </c>
       <c r="B234" t="n">
-        <v>0.008593750000000001</v>
+        <v>0.010546875</v>
       </c>
       <c r="C234" t="n">
-        <v>0.0029296875</v>
+        <v>0.0068359375</v>
       </c>
     </row>
     <row r="235">
@@ -3857,10 +3783,10 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>0.0044921875</v>
+        <v>0.005078125</v>
       </c>
       <c r="C235" t="n">
-        <v>0.003515625</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="236">
@@ -3870,10 +3796,10 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>0.003515625</v>
+        <v>0.003125</v>
       </c>
       <c r="C236" t="n">
-        <v>0.0015625</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="237">
@@ -3883,10 +3809,10 @@
         </is>
       </c>
       <c r="B237" t="n">
-        <v>0.0025390625</v>
+        <v>0.0009765625</v>
       </c>
       <c r="C237" t="n">
-        <v>0.0029296875</v>
+        <v>0.001953125</v>
       </c>
     </row>
     <row r="238">
@@ -3896,10 +3822,10 @@
         </is>
       </c>
       <c r="B238" t="n">
-        <v>0.012890625</v>
+        <v>0.0173828125</v>
       </c>
       <c r="C238" t="n">
-        <v>0.0041015625</v>
+        <v>0.0189453125</v>
       </c>
     </row>
     <row r="239">
@@ -3909,10 +3835,10 @@
         </is>
       </c>
       <c r="B239" t="n">
-        <v>0.0056640625</v>
+        <v>0.00546875</v>
       </c>
       <c r="C239" t="n">
-        <v>0.002734375</v>
+        <v>0.006640625</v>
       </c>
     </row>
     <row r="240">
@@ -3922,10 +3848,10 @@
         </is>
       </c>
       <c r="B240" t="n">
-        <v>0.0046875</v>
+        <v>0.0037109375</v>
       </c>
       <c r="C240" t="n">
-        <v>0.009375</v>
+        <v>0.0078125</v>
       </c>
     </row>
     <row r="241">
@@ -3935,10 +3861,10 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>0.003125</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C241" t="n">
-        <v>0.0078125</v>
+        <v>0.0052734375</v>
       </c>
     </row>
     <row r="242">
@@ -3948,10 +3874,10 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>0.0041015625</v>
+        <v>0.0013671875</v>
       </c>
       <c r="C242" t="n">
-        <v>0.00234375</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="243">
@@ -3961,10 +3887,10 @@
         </is>
       </c>
       <c r="B243" t="n">
+        <v>0.0013671875</v>
+      </c>
+      <c r="C243" t="n">
         <v>0.001953125</v>
-      </c>
-      <c r="C243" t="n">
-        <v>0.0037109375</v>
       </c>
     </row>
     <row r="244">
@@ -3974,10 +3900,10 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>0.0015625</v>
+        <v>0.001171875</v>
       </c>
       <c r="C244" t="n">
-        <v>0.0037109375</v>
+        <v>0.002734375</v>
       </c>
     </row>
     <row r="245">
@@ -3987,10 +3913,10 @@
         </is>
       </c>
       <c r="B245" t="n">
+        <v>0.000390625</v>
+      </c>
+      <c r="C245" t="n">
         <v>0.0021484375</v>
-      </c>
-      <c r="C245" t="n">
-        <v>0.0025390625</v>
       </c>
     </row>
     <row r="246">
@@ -4000,10 +3926,10 @@
         </is>
       </c>
       <c r="B246" t="n">
-        <v>0.001953125</v>
+        <v>0.0046875</v>
       </c>
       <c r="C246" t="n">
-        <v>0.0015625</v>
+        <v>0.00234375</v>
       </c>
     </row>
     <row r="247">
@@ -4016,7 +3942,7 @@
         <v>0.0025390625</v>
       </c>
       <c r="C247" t="n">
-        <v>0.0013671875</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="248">
@@ -4029,7 +3955,7 @@
         <v>0.00234375</v>
       </c>
       <c r="C248" t="n">
-        <v>0.0013671875</v>
+        <v>0.0033203125</v>
       </c>
     </row>
     <row r="249">
@@ -4039,10 +3965,10 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>0.00234375</v>
+        <v>0.00078125</v>
       </c>
       <c r="C249" t="n">
-        <v>0.001171875</v>
+        <v>0.0021484375</v>
       </c>
     </row>
     <row r="250">
@@ -4052,10 +3978,10 @@
         </is>
       </c>
       <c r="B250" t="n">
-        <v>0.00546875</v>
+        <v>0.003515625</v>
       </c>
       <c r="C250" t="n">
-        <v>0.003125</v>
+        <v>0.0029296875</v>
       </c>
     </row>
     <row r="251">
@@ -4068,7 +3994,7 @@
         <v>0.0037109375</v>
       </c>
       <c r="C251" t="n">
-        <v>0.0037109375</v>
+        <v>0.003125</v>
       </c>
     </row>
     <row r="252">
@@ -4078,10 +4004,10 @@
         </is>
       </c>
       <c r="B252" t="n">
+        <v>0.000390625</v>
+      </c>
+      <c r="C252" t="n">
         <v>0.0017578125</v>
-      </c>
-      <c r="C252" t="n">
-        <v>0.0037109375</v>
       </c>
     </row>
     <row r="253">
@@ -4091,10 +4017,10 @@
         </is>
       </c>
       <c r="B253" t="n">
+        <v>0.0005859375</v>
+      </c>
+      <c r="C253" t="n">
         <v>0.00234375</v>
-      </c>
-      <c r="C253" t="n">
-        <v>0.0015625</v>
       </c>
     </row>
     <row r="254">
@@ -4104,10 +4030,10 @@
         </is>
       </c>
       <c r="B254" t="n">
-        <v>0.003125</v>
+        <v>0.011328125</v>
       </c>
       <c r="C254" t="n">
-        <v>0.0013671875</v>
+        <v>0.0048828125</v>
       </c>
     </row>
     <row r="255">
@@ -4117,10 +4043,10 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>0.004296875</v>
+        <v>0.003515625</v>
       </c>
       <c r="C255" t="n">
-        <v>0.0005859375</v>
+        <v>0.0037109375</v>
       </c>
     </row>
     <row r="256">
@@ -4130,10 +4056,10 @@
         </is>
       </c>
       <c r="B256" t="n">
-        <v>0.0005859375</v>
+        <v>0.001171875</v>
       </c>
       <c r="C256" t="n">
-        <v>0.0015625</v>
+        <v>0.0017578125</v>
       </c>
     </row>
     <row r="257">
@@ -4143,10 +4069,23 @@
         </is>
       </c>
       <c r="B257" t="n">
-        <v>0.00078125</v>
+        <v>0.0005859375</v>
       </c>
       <c r="C257" t="n">
-        <v>0.001171875</v>
+        <v>0.0013671875</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="C258" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>